<commit_message>
add: git actions result with excel_reportv2
</commit_message>
<xml_diff>
--- a/reports/test_report2.xlsx
+++ b/reports/test_report2.xlsx
@@ -8821,7 +8821,7 @@
       </c>
       <c r="B26" s="30" t="inlineStr">
         <is>
-          <t>2026-04-16 04:29:42</t>
+          <t>2026-04-16 04:33:26</t>
         </is>
       </c>
       <c r="C26" s="32" t="n"/>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="B27" s="30" t="inlineStr">
         <is>
-          <t>tests/test_api.py</t>
+          <t>input/QFEapi.json</t>
         </is>
       </c>
       <c r="C27" s="32" t="n"/>
@@ -8869,7 +8869,7 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>42.3 초</t>
+          <t>2.594287157058716 초</t>
         </is>
       </c>
       <c r="C29" s="32" t="n"/>

</xml_diff>